<commit_message>
added data to choctaw Mississippi
</commit_message>
<xml_diff>
--- a/DawesRollsViewer/Dawes Rolls One Document/Choctaw/Mississippi Choctaw Newborn.xlsx
+++ b/DawesRollsViewer/Dawes Rolls One Document/Choctaw/Mississippi Choctaw Newborn.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="18">
   <si>
     <t>ID</t>
   </si>
@@ -59,6 +59,15 @@
   </si>
   <si>
     <t>Link</t>
+  </si>
+  <si>
+    <t>Mississippi Choctaw</t>
+  </si>
+  <si>
+    <t>Mississipi Blood New Born</t>
+  </si>
+  <si>
+    <t>Dawes Rolls Full Document - Choctaw By Blood - Page 168</t>
   </si>
 </sst>
 </file>
@@ -392,6 +401,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="11" max="11" width="25.42578125" customWidth="1"/>
+    <col min="12" max="12" width="28.28515625" customWidth="1"/>
+    <col min="14" max="14" width="53.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" t="s">
@@ -444,65 +459,207 @@
       <c r="A2">
         <v>1</v>
       </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2">
+        <v>168</v>
+      </c>
+      <c r="L2" t="s">
+        <v>16</v>
+      </c>
+      <c r="N2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
       </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3">
+        <v>168</v>
+      </c>
+      <c r="L3" t="s">
+        <v>16</v>
+      </c>
+      <c r="N3" t="str">
+        <f>N2</f>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4">
         <f t="shared" ref="A4:A12" si="0">A3+1</f>
         <v>3</v>
       </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4">
+        <v>168</v>
+      </c>
+      <c r="L4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" t="str">
+        <f t="shared" ref="N4:N12" si="1">N3</f>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5">
+        <v>168</v>
+      </c>
+      <c r="L5" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" t="str">
+        <f t="shared" si="1"/>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>168</v>
+      </c>
+      <c r="L6" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" t="str">
+        <f t="shared" si="1"/>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>168</v>
+      </c>
+      <c r="L7" t="s">
+        <v>16</v>
+      </c>
+      <c r="N7" t="str">
+        <f t="shared" si="1"/>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <v>168</v>
+      </c>
+      <c r="L8" t="s">
+        <v>16</v>
+      </c>
+      <c r="N8" t="str">
+        <f t="shared" si="1"/>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>168</v>
+      </c>
+      <c r="L9" t="s">
+        <v>16</v>
+      </c>
+      <c r="N9" t="str">
+        <f t="shared" si="1"/>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10">
+        <v>168</v>
+      </c>
+      <c r="L10" t="s">
+        <v>16</v>
+      </c>
+      <c r="N10" t="str">
+        <f t="shared" si="1"/>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11">
+        <v>168</v>
+      </c>
+      <c r="L11" t="s">
+        <v>16</v>
+      </c>
+      <c r="N11" t="str">
+        <f t="shared" si="1"/>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
+      </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12">
+        <v>168</v>
+      </c>
+      <c r="L12" t="s">
+        <v>16</v>
+      </c>
+      <c r="N12" t="str">
+        <f t="shared" si="1"/>
+        <v>Dawes Rolls Full Document - Choctaw By Blood - Page 168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>